<commit_message>
Act 3.2 — actualiza resultados, gráficas y golden test caso Sofía
Incluye reporte de avances regenerado, 6 figuras actualizadas,
breakdowns P2P/flujos y test de regresión del caso base de Sofía.
</commit_message>
<xml_diff>
--- a/resultados_comparacion.xlsx
+++ b/resultados_comparacion.xlsx
@@ -439,7 +439,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ganancia_neta_COP</t>
+          <t>Ganancia_neta_$</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -465,16 +465,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>150117.7782155001</v>
+        <v>149166.3554244795</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1126722937529999</v>
+        <v>0.9032746487033748</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0.9346750792679107</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1510131705234475</v>
+        <v>-0.1983322631223311</v>
       </c>
     </row>
     <row r="3">
@@ -484,16 +484,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>165409.7130091735</v>
+        <v>139838.4852193923</v>
       </c>
       <c r="C3" t="n">
-        <v>0.08849131417298814</v>
+        <v>0.5778404947855829</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7853866396558743</v>
+        <v>0.5979278960648478</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.2628055550044501</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="4">
@@ -503,16 +503,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>145202.5134603907</v>
+        <v>116457.2612184539</v>
       </c>
       <c r="C4" t="n">
-        <v>0.08849131417298814</v>
+        <v>0.5778404947855829</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7853866396558743</v>
+        <v>0.5979278960648478</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1602134241847393</v>
+        <v>-0.8991894959514061</v>
       </c>
     </row>
     <row r="5">
@@ -522,16 +522,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>135621.1514656016</v>
+        <v>104717.1460149028</v>
       </c>
       <c r="C5" t="n">
-        <v>0.08849131417298814</v>
+        <v>0.5778404947855829</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7853866396558743</v>
+        <v>0.5979278960648478</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1008841890743054</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="6">
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>129910.5786667173</v>
+        <v>103895.6403405108</v>
       </c>
       <c r="C6" t="n">
-        <v>0.08849131417298814</v>
+        <v>0.5778404947855829</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7853866396558743</v>
+        <v>0.5979278960648478</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.06136110830894741</v>
+        <v>-1</v>
       </c>
     </row>
   </sheetData>
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -606,19 +606,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>34243.97455063702</v>
+        <v>69557.69058363501</v>
       </c>
       <c r="C2" t="n">
-        <v>61607.21690378158</v>
+        <v>68766.10632519744</v>
       </c>
       <c r="D2" t="n">
-        <v>41400.01735499882</v>
+        <v>63733.32234452738</v>
       </c>
       <c r="E2" t="n">
-        <v>31818.65536020967</v>
+        <v>62647.42656579717</v>
       </c>
       <c r="F2" t="n">
-        <v>26108.0825613254</v>
+        <v>62179.90670261838</v>
       </c>
     </row>
     <row r="3">
@@ -628,19 +628,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>32297.31385398124</v>
+        <v>19171.76116172001</v>
       </c>
       <c r="C3" t="n">
-        <v>27554.99749148169</v>
+        <v>22737.72379661772</v>
       </c>
       <c r="D3" t="n">
-        <v>27554.99749148169</v>
+        <v>16134.25415423884</v>
       </c>
       <c r="E3" t="n">
-        <v>27554.99749148169</v>
+        <v>14165.09686728195</v>
       </c>
       <c r="F3" t="n">
-        <v>27554.99749148169</v>
+        <v>14072.01195558244</v>
       </c>
     </row>
     <row r="4">
@@ -650,19 +650,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>34678.53872393133</v>
+        <v>10632.28411977585</v>
       </c>
       <c r="C4" t="n">
-        <v>34678.53872393088</v>
+        <v>15272.55083458049</v>
       </c>
       <c r="D4" t="n">
-        <v>34678.53872393088</v>
+        <v>9133.044143474433</v>
       </c>
       <c r="E4" t="n">
-        <v>34678.53872393088</v>
+        <v>8538.463706013774</v>
       </c>
       <c r="F4" t="n">
-        <v>34678.53872393088</v>
+        <v>9200.804361307739</v>
       </c>
     </row>
     <row r="5">
@@ -672,19 +672,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29463.09716747679</v>
+        <v>46460.81498385874</v>
       </c>
       <c r="C5" t="n">
-        <v>26291.02206540454</v>
+        <v>33062.10426299668</v>
       </c>
       <c r="D5" t="n">
-        <v>26291.02206540454</v>
+        <v>21586.58297443768</v>
       </c>
       <c r="E5" t="n">
-        <v>26291.02206540454</v>
+        <v>19366.15887580989</v>
       </c>
       <c r="F5" t="n">
-        <v>26291.02206540454</v>
+        <v>18442.91732100224</v>
       </c>
     </row>
     <row r="6">
@@ -694,19 +694,41 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19434.85391947367</v>
+        <v>1664.661629266838</v>
       </c>
       <c r="C6" t="n">
-        <v>15277.93782457481</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>15277.93782457481</v>
+        <v>3396.302388271019</v>
       </c>
       <c r="E6" t="n">
-        <v>15277.93782457481</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>15277.93782457481</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1679.14294622309</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2473.755213504526</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -775,28 +797,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>0.9399999400338928</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.6686857048282192</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>-0.9999998871911312</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>5.640443442246002e-06</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>99.99999435955655</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>-372.2898112209105</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>-352.3681535425844</v>
       </c>
     </row>
     <row r="3">
@@ -804,28 +826,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>0.819999943655227</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.5802082045347263</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-0.9999999668484872</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1.657575637444197e-06</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>99.99999834242436</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>-280.1173348421868</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>-307.3849946240268</v>
       </c>
     </row>
     <row r="4">
@@ -833,28 +855,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>0.8199999436594572</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>0.6067446330092739</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>-0.9999999668470195</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1.657649028671462e-06</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>99.99999834235098</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>-294.2727143408214</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>-307.3849946254074</v>
       </c>
     </row>
     <row r="5">
@@ -862,28 +884,28 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>0.8199999436690311</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>0.6381509078540631</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>-0.9999999668445049</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1.657774758114215e-06</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>99.99999834222524</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>-309.5313015559924</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>-307.3849946286449</v>
       </c>
     </row>
     <row r="6">
@@ -891,28 +913,28 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>0.9399999400248249</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>0.9999999999999998</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>0.6933796137848025</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>-0.9999998871817479</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>5.640912613375778e-06</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>99.9999943590874</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>-383.5647415046785</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>-352.3681535376822</v>
       </c>
     </row>
     <row r="7">
@@ -920,28 +942,28 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>1.392088421217931</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>0.8865130594912339</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>-0.5225055042848792</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>23.87472478575604</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>76.12527521424396</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>-745.9715435404396</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>-408.547157976501</v>
       </c>
     </row>
     <row r="8">
@@ -949,28 +971,28 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>1.417903162479265</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.9496111253101039</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>0.9999999999999998</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>-1612.767297759848</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>-410.7494349483037</v>
       </c>
     </row>
     <row r="9">
@@ -978,28 +1000,28 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1.496962380900113</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>0.913543094052895</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>-0.762286730110183</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>11.88566349449085</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>88.11433650550916</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>-1030.530138898106</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>-334.1509424896282</v>
       </c>
     </row>
     <row r="10">
@@ -1007,28 +1029,28 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1.823122656166763</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.9048772389131633</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>-0.4470690083572017</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>27.64654958213992</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>72.35345041786007</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>-640.9005166264891</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>-370.7146991209874</v>
       </c>
     </row>
     <row r="11">
@@ -1036,28 +1058,28 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>3.532530847396926</v>
+        <v>2.237950589074116</v>
       </c>
       <c r="C11" t="n">
-        <v>0.2306358242409365</v>
+        <v>0.9299434223848493</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0562833676369127</v>
+        <v>0.4489013975025599</v>
       </c>
       <c r="F11" t="n">
-        <v>47.18583161815436</v>
+        <v>72.445069875128</v>
       </c>
       <c r="G11" t="n">
-        <v>52.81416838184563</v>
+        <v>27.554930124872</v>
       </c>
       <c r="H11" t="n">
-        <v>-486.2362905051125</v>
+        <v>-235.9398716672053</v>
       </c>
       <c r="I11" t="n">
-        <v>1209.376275252651</v>
+        <v>98.05096264762204</v>
       </c>
     </row>
     <row r="12">
@@ -1065,28 +1087,28 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>8.266650006244634</v>
+        <v>3.439461603981111</v>
       </c>
       <c r="C12" t="n">
-        <v>0.3033029825583616</v>
+        <v>0.9020098936947899</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5447138968193286</v>
+        <v>0.3700826874666402</v>
       </c>
       <c r="F12" t="n">
-        <v>77.23569484096643</v>
+        <v>68.50413437333201</v>
       </c>
       <c r="G12" t="n">
-        <v>22.76430515903357</v>
+        <v>31.49586562666799</v>
       </c>
       <c r="H12" t="n">
-        <v>-1157.494114958183</v>
+        <v>-400.8616662481227</v>
       </c>
       <c r="I12" t="n">
-        <v>1120.966733563085</v>
+        <v>-74.41598735084293</v>
       </c>
     </row>
     <row r="13">
@@ -1094,28 +1116,28 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>10.11358862402805</v>
+        <v>4.10301821050562</v>
       </c>
       <c r="C13" t="n">
-        <v>0.3322949008468301</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>0.9791783607854583</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4450400887456926</v>
+        <v>0.5335703135392378</v>
       </c>
       <c r="F13" t="n">
-        <v>72.25200443728464</v>
+        <v>76.67851567696188</v>
       </c>
       <c r="G13" t="n">
-        <v>27.74799556271537</v>
+        <v>23.32148432303811</v>
       </c>
       <c r="H13" t="n">
-        <v>-1425.423635533201</v>
+        <v>-489.513598027426</v>
       </c>
       <c r="I13" t="n">
-        <v>916.9385802818665</v>
+        <v>-57.16303604939945</v>
       </c>
     </row>
     <row r="14">
@@ -1123,28 +1145,28 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>11.59034282110254</v>
+        <v>3.679416446228168</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3938301517104429</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0.8970576253933392</v>
       </c>
       <c r="E14" t="n">
-        <v>0.06279997838788981</v>
+        <v>0.6161853741023305</v>
       </c>
       <c r="F14" t="n">
-        <v>53.13999891939449</v>
+        <v>80.80926870511652</v>
       </c>
       <c r="G14" t="n">
-        <v>46.86000108060551</v>
+        <v>19.19073129488347</v>
       </c>
       <c r="H14" t="n">
-        <v>-1642.073825936403</v>
+        <v>-395.4822538578713</v>
       </c>
       <c r="I14" t="n">
-        <v>484.4319868237744</v>
+        <v>36.50989633551531</v>
       </c>
     </row>
     <row r="15">
@@ -1152,28 +1174,28 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>11.38772509545866</v>
+        <v>4.276429554510765</v>
       </c>
       <c r="C15" t="n">
-        <v>0.4111881536261818</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>0.9294215164577244</v>
       </c>
       <c r="E15" t="n">
-        <v>0.07378912408210732</v>
+        <v>0.5016611875080279</v>
       </c>
       <c r="F15" t="n">
-        <v>53.68945620410537</v>
+        <v>75.08305937540139</v>
       </c>
       <c r="G15" t="n">
-        <v>46.31054379589464</v>
+        <v>24.9169406245986</v>
       </c>
       <c r="H15" t="n">
-        <v>-1612.215511418181</v>
+        <v>-517.0999052847625</v>
       </c>
       <c r="I15" t="n">
-        <v>403.4630157730165</v>
+        <v>-131.920529389885</v>
       </c>
     </row>
     <row r="16">
@@ -1181,28 +1203,28 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>7.842862055010452</v>
+        <v>4.350745143257377</v>
       </c>
       <c r="C16" t="n">
-        <v>0.2878037006788998</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0.98138060402169</v>
       </c>
       <c r="E16" t="n">
-        <v>0.04819942791556583</v>
+        <v>0.5009141549904218</v>
       </c>
       <c r="F16" t="n">
-        <v>52.4099713957783</v>
+        <v>75.04570774952109</v>
       </c>
       <c r="G16" t="n">
-        <v>47.59002860422171</v>
+        <v>24.9542922504789</v>
       </c>
       <c r="H16" t="n">
-        <v>-1096.448802051681</v>
+        <v>-569.8999782549944</v>
       </c>
       <c r="I16" t="n">
-        <v>646.9796104832997</v>
+        <v>-119.0252889707308</v>
       </c>
     </row>
     <row r="17">
@@ -1210,28 +1232,28 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>1.880353385306708</v>
+        <v>3.358229955435879</v>
       </c>
       <c r="C17" t="n">
-        <v>0.1878771421528856</v>
+        <v>0.8816705225208304</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.06116695464953887</v>
+        <v>0.8050010926168463</v>
       </c>
       <c r="F17" t="n">
-        <v>46.94165226752306</v>
+        <v>90.25005463084231</v>
       </c>
       <c r="G17" t="n">
-        <v>53.05834773247695</v>
+        <v>9.749945369157679</v>
       </c>
       <c r="H17" t="n">
-        <v>-257.2683742379943</v>
+        <v>-445.5088447732496</v>
       </c>
       <c r="I17" t="n">
-        <v>1033.542712981327</v>
+        <v>191.0635893751935</v>
       </c>
     </row>
     <row r="18">
@@ -1239,28 +1261,28 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>2.020003288577634</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>0.936418766552147</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>-0.4545285352714353</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>27.27357323642823</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>72.72642676357177</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>-294.4701895372156</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>-293.4866547539098</v>
       </c>
     </row>
     <row r="19">
@@ -1268,28 +1290,28 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>0.572732682271398</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>0.8137926067306609</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>0.6735662474513869</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>83.67831237256935</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>16.32168762743066</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>-54.69000408611848</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>389.1339941172304</v>
       </c>
     </row>
     <row r="20">
@@ -1297,28 +1319,28 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>0.6446942833678948</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>0.6971857962676258</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>0.5555998764593696</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>77.77999382296848</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>22.22000617703152</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>-81.04701299952464</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>234.3017010337495</v>
       </c>
     </row>
     <row r="21">
@@ -1326,28 +1348,28 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>0.8776155650537559</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>0.5419237956168438</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>0.4581106084246955</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>72.90553042123477</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>27.09446957876522</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>-110.4286908828075</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>50.09677675034703</v>
       </c>
     </row>
     <row r="22">
@@ -1355,28 +1377,28 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>0.7395662405520669</v>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>0.6212167895658525</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>0.7624415905876064</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>88.12207952938031</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>11.87792047061968</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>-93.01355269698928</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>124.5049810738735</v>
       </c>
     </row>
     <row r="23">
@@ -1384,28 +1406,28 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>0</v>
+        <v>1.541227153157251</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>0.820163757030747</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>-0.9999999717508008</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1.412459960844969e-06</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>99.99999858754005</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>-601.1563832675619</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>-577.7440656052258</v>
       </c>
     </row>
     <row r="24">
@@ -1413,28 +1435,28 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>1.083138434494439</v>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>0.8981739860870275</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>-0.7996195567157519</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>10.0190221642124</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>89.9809778357876</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>-339.5742514868742</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>-369.0338071114764</v>
       </c>
     </row>
     <row r="25">
@@ -1442,28 +1464,28 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>1.059999935996569</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>0.9999999999999998</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>0.7650368998564695</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>-0.9999998641819269</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>6.790903660779226e-06</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>99.99999320909635</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>-462.2653405584261</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>-397.3513192799177</v>
       </c>
     </row>
   </sheetData>
@@ -1483,7 +1505,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PoF_P2P_vs_C4</t>
+          <t>RPE_P2P_vs_C4</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -1514,19 +1536,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.1346089702964729</v>
+        <v>0.3034914606255735</v>
       </c>
       <c r="B2" t="n">
-        <v>20.3411259094923</v>
+        <v>14.16391272090346</v>
       </c>
       <c r="C2" t="n">
-        <v>-7677.160554640755</v>
+        <v>-10760.89694391862</v>
       </c>
       <c r="D2" t="n">
-        <v>5815.69891515902</v>
+        <v>-4047.532312671623</v>
       </c>
       <c r="E2" t="n">
-        <v>-1861.461639481735</v>
+        <v>-14808.42925659025</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>

</xml_diff>